<commit_message>
sheet job name change
</commit_message>
<xml_diff>
--- a/job-filters.xlsx
+++ b/job-filters.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Shubham\fiverr\raikaphotograph\task-schedular\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F3C3DEF-5351-4C46-9DFB-D98DB787BA12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B80AD671-5530-4DB7-80CF-991463D768BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="43">
   <si>
     <t>Job Name</t>
   </si>
@@ -273,6 +273,9 @@
 Inside Sales Executive
 Sales Manager
 BPO Executive</t>
+  </si>
+  <si>
+    <t>photographer assistant</t>
   </si>
 </sst>
 </file>
@@ -710,9 +713,9 @@
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="1:12" ht="201.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:12" ht="187.2" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>13</v>
+        <v>42</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>14</v>

</xml_diff>